<commit_message>
added 2 more leads
</commit_message>
<xml_diff>
--- a/output/workbooks/GenosAI_OrganicLeads.xlsx
+++ b/output/workbooks/GenosAI_OrganicLeads.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1805,6 +1805,172 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Home Seekers</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Thomas Potgieter</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; Managing Director</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>info@homeseeker.co.za</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>+27 012 880 3127</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.homeseeker.co.za/</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/thomas-potgieter-a4972b96/</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Pretoria</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Gauteng, South Africa</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Organic/Manual</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Pending Send</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>HomeSeeker_Audit_GenosAI.pptx</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp AI for buyer inquiries (24/7 response + viewing booking); lead routing from Property24/Private Property to agents; FICA compliance document collection workflow; agent recruitment intake automation (agents.homeseeker.co.za); buyer nurture drip for non-converting inquiries; post-sale review request sequence</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>Fixed-fee platform — agents keep 100% commission. Founded 2025. 416+ active listings. Ice-breaker: Rode Potgieter 8 deals / R11.44M Oct 2025 (LinkedIn). Co-LinkedIn: linkedin.com/company/home-seekers-sa</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Swisszaco Estates</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>+2348101658350</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://swisszacoestates.com/</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/swisscazo-estate/about/</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate Development</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Organic/LinkedIn</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Contact TBD — LinkedIn Pending</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>output/decks/SwisszacoEstates_Audit_GenosAI.pptx</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp AI buyer agent (property inquiry + site visit booking); agent network recruitment automation (intake, onboarding, nurture); lead nurture sequences (re-engagement + new listing alerts); post-handover review and testimonial collection; diaspora investor nurture (UK/US/Canada) via WhatsApp</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>Contact TBD — outreach via company LinkedIn page. Score 3/10, HIGH priority.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1817,7 +1983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2379,6 +2545,105 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Home Seekers</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Thomas Potgieter</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>info@homeseeker.co.za</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>416 listings and buyer inquiries waiting while agents are at viewings</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Hi Thomas,
+Saw the LinkedIn post on Rode's October run — 8 deals for R11.44M on a 100%-commission model. That number makes the platform's value proposition more credible than any recruitment copy.
+The question it raised for me: when a buyer submits an inquiry on one of your 416 listings at 9pm on a Sunday, what happens to that lead before Monday morning? In South Africa's market, that buyer has already sent the same inquiry to three other agents on Property24. The one who responds on WhatsApp first — even if it's an AI — controls the conversation.
+Genos AI builds WhatsApp automation specifically for real estate platforms. For HomeSeeker's model:
+WhatsApp AI for buyer inquiries — responds 24/7, answers property questions, qualifies budget and timeline, books the viewing without the agent being online. Lead goes from Property24 to confirmed appointment automatically.
+Lead routing by area and type — inquiry captured via WhatsApp, AI qualifies the buyer, assigns to the right agent based on property type and location, logged in your system.
+FICA and compliance document collection — for your back-office platform, an AI workflow that requests, follows up, and confirms receipt of required documents from buyers and sellers. Agents stop chasing paper manually.
+Agent recruitment intake — agents.homeseeker.co.za gets an AI that screens applicants, asks qualifying questions, and schedules intro calls. You're not reading every enquiry manually.
+I'm Rohan Malik, CEO of Genos AI. We build AI automation for real estate operations — WhatsApp agents, lead qualification flows, compliance automations. Happy to show you how it works in 20 minutes.
+Rohan Malik
+CEO, Genos AI
++91 638-714-2699  |  hello@genosai.tech  |  www.genosai.tech</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Hi Thomas, following up on my last message. The core gap — buyer inquiries on your 416 listings sitting unanswered while agents are at viewings — is the fastest to close. A WhatsApp AI agent for Home Seekers is typically live in under 2 weeks. Happy to walk through it in 20 minutes. — Rohan | Genos AI</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Thomas, last one from me. On a 100%-commission platform, an agent's income depends entirely on their lead conversion speed. An AI that ensures no buyer inquiry goes unanswered — even at 9pm on a Sunday — is the infrastructure that makes your agents more productive than any franchise competitor. Leaving this here if the timing isn't right. — Rohan | Genos AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Swisszaco Estates</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Swisszaco's agent network and a property inquiry process still stuck on contact forms</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Hi,
+Came across Swisszaco Estates while researching real estate developers in Nigeria. CAC-registered since March 2012 — 13 years in the market across construction, estate development, architectural design, and urban development. The agent network program stood out as an indicator the business is actively scaling.
+One gap that showed up immediately on swisszacoestates.com: there's no way for a property buyer or investor to get a fast response outside business hours. The contact form is the only entry point — no chat widget, no WhatsApp integration, no booking flow for property viewings. In the Nigerian market, where most buyers are comparing 3-4 developers simultaneously and expect a WhatsApp reply within the hour, a contact form with a 24-48 hour turnaround quietly hands those leads to whoever responds first.
+The same applies to your agent network. Agents researching whether to join need immediate answers on commission structure, available projects, and onboarding — a contact form puts that decision on hold.
+What we build for real estate developers at Genos AI: WhatsApp AI agents that qualify buyers (property type, location, budget, timeline), book site visits automatically, and route hot leads to the right agent — 24/7, no manual handling. We also build agent recruitment flows that capture and nurture new agent sign-ups without your team chasing each one.
+I'm Rohan Malik, CEO of Genos AI. Did a full audit of swisszacoestates.com — happy to share it or walk through it in 15 minutes.
+Rohan Malik
+CEO, Genos AI
++91 638-714-2699  |  hello@genosai.tech  |  www.genosai.tech</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Hi, following up on my last message. The core gap — property inquiries hitting a static contact form while competitors respond on WhatsApp in minutes — is the fastest thing to fix. A WhatsApp AI agent for Swisszaco is typically live within 2 weeks. Happy to show you exactly how it works in 15 minutes. — Rohan | Genos AI</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Last one from me. The Swisszaco audit covers the WhatsApp buyer qualification flow, agent recruitment automation, and the property viewing booking system specifically. If the timing isn't right, no problem — leaving it here in case it's useful later. — Rohan | Genos AI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2391,7 +2656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2854,6 +3119,98 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Home Seekers</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Thomas Potgieter</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>info@homeseeker.co.za</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Email Pending</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Send cold email — pitch AI automation</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Swisszaco Estates</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Real Estate Development</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Contact TBD</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Source contact via LinkedIn — send cold email + deck</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>$3,000 - $6,000</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>